<commit_message>
add code for n-grams
</commit_message>
<xml_diff>
--- a/fig/learn/gi_freq.xlsx
+++ b/fig/learn/gi_freq.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t>Word</t>
   </si>
@@ -28,96 +28,171 @@
     <t>male</t>
   </si>
   <si>
+    <t>as</t>
+  </si>
+  <si>
+    <t>and</t>
+  </si>
+  <si>
+    <t>nonbinary</t>
+  </si>
+  <si>
+    <t>not</t>
+  </si>
+  <si>
+    <t>demigirl</t>
+  </si>
+  <si>
+    <t>agender genderfluid</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>dont</t>
+  </si>
+  <si>
+    <t>im</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>is</t>
+  </si>
+  <si>
+    <t>this</t>
+  </si>
+  <si>
+    <t>question</t>
+  </si>
+  <si>
+    <t>transmasculine</t>
+  </si>
+  <si>
+    <t>unsure</t>
+  </si>
+  <si>
+    <t>demiboy</t>
+  </si>
+  <si>
+    <t>the</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>there</t>
+  </si>
+  <si>
+    <t>theythem</t>
+  </si>
+  <si>
+    <t>girl</t>
+  </si>
+  <si>
+    <t>one</t>
+  </si>
+  <si>
+    <t>change</t>
+  </si>
+  <si>
+    <t>that</t>
+  </si>
+  <si>
+    <t>be</t>
+  </si>
+  <si>
+    <t>man</t>
+  </si>
+  <si>
+    <t>at</t>
+  </si>
+  <si>
+    <t>woman</t>
+  </si>
+  <si>
+    <t>genderqueer</t>
+  </si>
+  <si>
+    <t>to</t>
+  </si>
+  <si>
+    <t>guy</t>
+  </si>
+  <si>
+    <t>identify</t>
+  </si>
+  <si>
+    <t>was born</t>
+  </si>
+  <si>
+    <t>but also</t>
+  </si>
+  <si>
     <t>agender</t>
   </si>
   <si>
-    <t>nonbinary</t>
-  </si>
-  <si>
-    <t>demigirl</t>
-  </si>
-  <si>
-    <t>gender</t>
-  </si>
-  <si>
-    <t>question</t>
-  </si>
-  <si>
-    <t>transmasculine</t>
-  </si>
-  <si>
-    <t>unsure</t>
-  </si>
-  <si>
-    <t>demiboy</t>
-  </si>
-  <si>
-    <t>time</t>
-  </si>
-  <si>
-    <t>theythem</t>
-  </si>
-  <si>
-    <t>born</t>
-  </si>
-  <si>
-    <t>girl</t>
-  </si>
-  <si>
-    <t>one</t>
-  </si>
-  <si>
-    <t>change</t>
-  </si>
-  <si>
-    <t>man</t>
-  </si>
-  <si>
-    <t>woman</t>
-  </si>
-  <si>
-    <t>genderqueer</t>
-  </si>
-  <si>
-    <t>guy</t>
-  </si>
-  <si>
     <t>unknown</t>
   </si>
   <si>
     <t>hombre</t>
   </si>
   <si>
+    <t>jewish</t>
+  </si>
+  <si>
     <t>androgyne</t>
   </si>
   <si>
     <t>know</t>
   </si>
   <si>
-    <t>confused</t>
-  </si>
-  <si>
     <t>nonconforming</t>
   </si>
   <si>
     <t>identity</t>
   </si>
   <si>
-    <t>idea</t>
+    <t>misogynistic</t>
+  </si>
+  <si>
+    <t>homophobic</t>
+  </si>
+  <si>
+    <t>can</t>
+  </si>
+  <si>
+    <t>should</t>
   </si>
   <si>
     <t>transfemme</t>
   </si>
   <si>
+    <t>who</t>
+  </si>
+  <si>
     <t>acts</t>
   </si>
   <si>
-    <t>called</t>
+    <t>put</t>
+  </si>
+  <si>
+    <t>but</t>
   </si>
   <si>
     <t>mostly</t>
   </si>
   <si>
+    <t>also</t>
+  </si>
+  <si>
+    <t>so</t>
+  </si>
+  <si>
+    <t>only</t>
+  </si>
+  <si>
     <t>hehim</t>
   </si>
   <si>
@@ -133,6 +208,9 @@
     <t>dude</t>
   </si>
   <si>
+    <t>himalpha</t>
+  </si>
+  <si>
     <t>bigender</t>
   </si>
   <si>
@@ -142,6 +220,9 @@
     <t>questioning</t>
   </si>
   <si>
+    <t>for</t>
+  </si>
+  <si>
     <t>fluid</t>
   </si>
   <si>
@@ -154,25 +235,91 @@
     <t>transmasc</t>
   </si>
   <si>
-    <t>straight</t>
+    <t>attack helicopter</t>
+  </si>
+  <si>
+    <t>rocket ship</t>
+  </si>
+  <si>
+    <t>drop table</t>
+  </si>
+  <si>
+    <t>table responses</t>
+  </si>
+  <si>
+    <t>pretty confused</t>
+  </si>
+  <si>
+    <t>confused most</t>
+  </si>
+  <si>
+    <t>most of</t>
+  </si>
+  <si>
+    <t>such thing</t>
+  </si>
+  <si>
+    <t>very idea</t>
   </si>
   <si>
     <t>masculine sheher</t>
   </si>
   <si>
+    <t>nigger killer</t>
+  </si>
+  <si>
+    <t>relevant meant</t>
+  </si>
+  <si>
+    <t>on last</t>
+  </si>
+  <si>
+    <t>belive in</t>
+  </si>
+  <si>
+    <t>mentally ill</t>
+  </si>
+  <si>
+    <t>ill shit</t>
+  </si>
+  <si>
+    <t>shit uncertain</t>
+  </si>
+  <si>
     <t>uncertain idk</t>
   </si>
   <si>
+    <t>idk what</t>
+  </si>
+  <si>
+    <t>what its</t>
+  </si>
+  <si>
+    <t>its called</t>
+  </si>
+  <si>
     <t>feel somewhat</t>
   </si>
   <si>
     <t>somewhat feminine</t>
   </si>
   <si>
+    <t>feminine here</t>
+  </si>
+  <si>
+    <t>stupid stuff</t>
+  </si>
+  <si>
     <t>femalenonbinary two</t>
   </si>
   <si>
     <t>two spirit</t>
+  </si>
+  <si>
+    <t>bullshit ass</t>
+  </si>
+  <si>
+    <t>am straight</t>
   </si>
 </sst>
 </file>
@@ -530,7 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -546,7 +693,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -570,7 +717,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -586,7 +733,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -594,7 +741,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -602,7 +749,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -610,7 +757,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -618,7 +765,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -626,7 +773,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -634,7 +781,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -642,7 +789,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -650,7 +797,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -658,7 +805,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -706,7 +853,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -714,7 +861,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -722,7 +869,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -730,7 +877,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -738,7 +885,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -746,7 +893,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -754,7 +901,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2">
@@ -762,7 +909,7 @@
         <v>29</v>
       </c>
       <c r="B29">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -770,7 +917,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -778,7 +925,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -786,7 +933,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -794,7 +941,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -802,7 +949,7 @@
         <v>34</v>
       </c>
       <c r="B34">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -810,7 +957,7 @@
         <v>35</v>
       </c>
       <c r="B35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2">
@@ -818,7 +965,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -826,7 +973,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -946,6 +1093,398 @@
         <v>52</v>
       </c>
       <c r="B52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>53</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>54</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
+        <v>55</v>
+      </c>
+      <c r="B55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
+        <v>56</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
+        <v>57</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
+        <v>58</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
+        <v>59</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
+        <v>60</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>61</v>
+      </c>
+      <c r="B61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>64</v>
+      </c>
+      <c r="B64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
+        <v>65</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" t="s">
+        <v>66</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" t="s">
+        <v>67</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
+        <v>68</v>
+      </c>
+      <c r="B68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
+        <v>69</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
+        <v>70</v>
+      </c>
+      <c r="B70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" t="s">
+        <v>71</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
+        <v>72</v>
+      </c>
+      <c r="B72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
+        <v>73</v>
+      </c>
+      <c r="B73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
+        <v>74</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
+        <v>75</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" t="s">
+        <v>76</v>
+      </c>
+      <c r="B76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" t="s">
+        <v>77</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
+        <v>78</v>
+      </c>
+      <c r="B78">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
+        <v>79</v>
+      </c>
+      <c r="B79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
+        <v>80</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>81</v>
+      </c>
+      <c r="B81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>82</v>
+      </c>
+      <c r="B82">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" t="s">
+        <v>83</v>
+      </c>
+      <c r="B83">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" t="s">
+        <v>84</v>
+      </c>
+      <c r="B84">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
+        <v>85</v>
+      </c>
+      <c r="B85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
+        <v>86</v>
+      </c>
+      <c r="B86">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" t="s">
+        <v>87</v>
+      </c>
+      <c r="B87">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" t="s">
+        <v>88</v>
+      </c>
+      <c r="B88">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
+        <v>89</v>
+      </c>
+      <c r="B89">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
+        <v>90</v>
+      </c>
+      <c r="B90">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>91</v>
+      </c>
+      <c r="B91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>92</v>
+      </c>
+      <c r="B92">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>93</v>
+      </c>
+      <c r="B93">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
+        <v>94</v>
+      </c>
+      <c r="B94">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>95</v>
+      </c>
+      <c r="B95">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>96</v>
+      </c>
+      <c r="B96">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
+        <v>97</v>
+      </c>
+      <c r="B97">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" t="s">
+        <v>98</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
+        <v>99</v>
+      </c>
+      <c r="B99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
+        <v>100</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" t="s">
+        <v>101</v>
+      </c>
+      <c r="B101">
         <v>1</v>
       </c>
     </row>

</xml_diff>